<commit_message>
scale up scrape + relax llm filter for nigeria x creators (100-150 per creator)
</commit_message>
<xml_diff>
--- a/Scraped Tweets - Nigeria/Agba John Doe_scope_relevant.xlsx
+++ b/Scraped Tweets - Nigeria/Agba John Doe_scope_relevant.xlsx
@@ -14,15 +14,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="121">
   <si>
     <t>text</t>
   </si>
   <si>
-    <t>no guarantee that the woman you'll marry wasn't one. It is your personal decision. Lastly, I've always said that three things keep &amp;amp; sustain marriages. 1) kindness 2) selflessness 3) deliberate commitment If a former prostitute wants her marriage to work, she'll deliberately</t>
-  </si>
-  <si>
-    <t>Provision will act as a shield for you as a man &amp;amp; husband. Without it, you're completely "naked". No woman will sympathize with you, for too long. Never delegate that role to her. Else, she will see you as useless. And you'll be forced to play by her own rules. End.</t>
+    <t>no guarantee that the woman you'll marry wasn't one. It is your personal decision. Lastly, I've always said that three things keep &amp; sustain marriages. 1) kindness 2) selflessness 3) deliberate commitment If a former prostitute wants her marriage to work, she'll deliberately</t>
+  </si>
+  <si>
+    <t>Provision will act as a shield for you as a man &amp; husband. Without it, you're completely "naked". No woman will sympathize with you, for too long. Never delegate that role to her. Else, she will see you as useless. And you'll be forced to play by her own rules. End.</t>
   </si>
   <si>
     <t>Don't be a REAL man.</t>
@@ -46,55 +46,112 @@
     <t>his wife's inactive poison. Money, is not required to find a wife. But when children start coming in, money is one important element, that will help a man sustain his marriage, and earn his respect and submission. Women do NOT like paying bills. Even if they have the means</t>
   </si>
   <si>
+    <t>It's my wish, that young single men read the DMs I'll share tonight. A young man that is cohabiting with his fiancée, sent me a very brilliant submission from what he has learnt &amp; what he has been doing. You'll not get what you're learning from here, anywhere else on SM. End.</t>
+  </si>
+  <si>
+    <t>thread, wicked. They think they'll do better. Do you think that if those men thought their wives would be wicked to them in future, they would have agreed to marry them? Some years into my marriage, I became jobless. Despite my wife not making me feel disrespected, I was</t>
+  </si>
+  <si>
     <t>the men remain in the "dark". Let's not pretend. Every man wants to believe that his wife is a "Saint". And a Saint she will remain, until you unearth that which she thought would never be known. So for me, a former prostitute or hook up girl can make a good wife or mother.</t>
   </si>
   <si>
+    <t>All those women that sexualise themselves publicly, are bad women. They don't deserve to get married, neither do they deserve to be mothers. You'll be punishing your innocent children, if you let any of them come through such women. Your children deserve better. End.</t>
+  </si>
+  <si>
     <t>If I decide to look at my own marriage, and all I've been experiencing in it, you'll hardly see me come here to paint the negative sides of marriage. But I'll never do that because I've refused to see myself as an exception. With the grace of God and man, I've been leading my</t>
   </si>
   <si>
-    <t>who doesn't know her story will not find her worthy to be a wife &amp;amp; mother to his kids? Remember, I had said that a woman will treat you like a king until you discover her secrets? That's exactly what is playing out in a lot of marriages where the men married women like that &amp;amp;</t>
-  </si>
-  <si>
-    <t>When men with experience talk, young &amp;amp; inexperienced men will just be spewing gibberish. Look at this DM from a divorced man. Just this morning, I said a man should not buy a property in the name of his wife &amp;amp; a wife (if given permission), should not buy a property in her</t>
-  </si>
-  <si>
-    <t>if he knew &amp;amp; still decided to marry her. Men &amp;amp; Women commit the same crimes, but we do not go to the same prison. Neither do we do same time. It's men who patronize these prostitutes. It's still men that will marry them. Even if you as a man, never patronized one, it's</t>
-  </si>
-  <si>
-    <t>nothing is guaranteed outside. Don't punish her by making her a divorcee because it will be tougher on her &amp;amp; make her life miserable. God will not forgive you, for hurting a woman that opened up her heart to you &amp;amp; willingly accepted to submit to you. Lastly, if your father is</t>
+    <t>who doesn't know her story will not find her worthy to be a wife &amp; mother to his kids? Remember, I had said that a woman will treat you like a king until you discover her secrets? That's exactly what is playing out in a lot of marriages where the men married women like that &amp;</t>
+  </si>
+  <si>
+    <t>if he knew &amp; still decided to marry her. Men &amp; Women commit the same crimes, but we do not go to the same prison. Neither do we do same time. It's men who patronize these prostitutes. It's still men that will marry them. Even if you as a man, never patronized one, it's</t>
+  </si>
+  <si>
+    <t>When men with experience talk, young &amp; inexperienced men will just be spewing gibberish. Look at this DM from a divorced man. Just this morning, I said a man should not buy a property in the name of his wife &amp; a wife (if given permission), should not buy a property in her</t>
   </si>
   <si>
     <t>And a real man is woman's mole. End.</t>
   </si>
   <si>
+    <t>nothing is guaranteed outside. Don't punish her by making her a divorcee because it will be tougher on her &amp; make her life miserable. God will not forgive you, for hurting a woman that opened up her heart to you &amp; willingly accepted to submit to you. Lastly, if your father is</t>
+  </si>
+  <si>
+    <t>family, well. But all that can change if things go south, and remain so, for a very very long time. A wife is the most amazing wife, is because her husband has been fortunate with life. A husband has been the most amazing husband is because he has been fortunate not to trigger</t>
+  </si>
+  <si>
     <t>Women, Will you support your sons or brothers, if they wish to marry a lady raised by a single mother, through divorce. Or a single mother who is divorced or never married? Vote and/or comment. Men, use the see result option.</t>
   </si>
   <si>
+    <t>3. He married into a wealthy family. His business crashed, and his wife moved out. 3 years of marriage, about to crash.</t>
+  </si>
+  <si>
     <t>become too comfortable as a man. Why? Because you expect your wife to love you. You'll be disappointed in the long run. And the sad part of all these, is that women will always think that they're different from other women. They don't know what they're capable of doing,</t>
   </si>
   <si>
-    <t>I just feel "sorry" for my children. Everything they will ever hear from me &amp;amp; my wife, will be the complete opposite of what they read and see on social media. They'll so hate me &amp;amp; their mother, but I hope God will see our conscience &amp;amp; reveal to them that we meant well. End.</t>
-  </si>
-  <si>
-    <t>emotional and because you, as the man, has a soft spot for her, you fail to recognize when she's being manipulative. And the more you keep falling for it, the more trouble you're building up for the future. Stand firm when it's necessary &amp;amp; let her know that yes you care for</t>
+    <t>I just feel "sorry" for my children. Everything they will ever hear from me &amp; my wife, will be the complete opposite of what they read and see on social media. They'll so hate me &amp; their mother, but I hope God will see our conscience &amp; reveal to them that we meant well. End.</t>
+  </si>
+  <si>
+    <t>My wife doesn't love me. She respects and submits to me. Stop looking for women that will love you. Find one that will appreciate your worth, has good character and can help you raise responsible children. And be there for you, when you're old &amp; frail. End</t>
+  </si>
+  <si>
+    <t>6. Remember my earlier tweet of a young man that is cohabiting with his fiancée? Make sure you read this and learn.</t>
+  </si>
+  <si>
+    <t>emotional and because you, as the man, has a soft spot for her, you fail to recognize when she's being manipulative. And the more you keep falling for it, the more trouble you're building up for the future. Stand firm when it's necessary &amp; let her know that yes you care for</t>
+  </si>
+  <si>
+    <t>I also got another beautiful one. His wife has been the one taking care of the bills for over 2 years. And she acts as if he's the one paying all the bills and shows him respect and submission. He's happy he married a wonderful wife. But hopes God changes his situation. End.</t>
+  </si>
+  <si>
+    <t>11. Married for almost 3 years, without any job or reasonable side hustle. His wife has been in charge of all the bills. According to him, she's the best wife ever. Read!</t>
   </si>
   <si>
     <t>Call it whatever you may. Your wife must always feel that she needs you. She must feel that she's with you for a purpose, she may not get elsewhere. No matter how small. Not all men are equally rich/famous. But their wives still respect them. This's nature, not theory. End</t>
   </si>
   <si>
-    <t>Please keep all relationship or marriage matters until inec declares the result of the elections. My children deserve a good country to grow in. We need a good country before we can be emotionally balanced to love &amp;amp; be happy in it. End.</t>
-  </si>
-  <si>
-    <t>that we have equal amount of men and women in this community. It clearly says one thing... The pain of heartbreak is more on the one who loves &amp;amp; provides. Women are very unapologetic when they want to move on. And that's how they are created. But you won't listen. End.</t>
-  </si>
-  <si>
-    <t>Nothing is as disappointing to a lady that's trying to make ends meet, &amp;amp; do so legitimately, seeing another lady that is making ends meet, by just opening her legs. This is why they call such ladies "P. ick Mes" They feel no man wants them. In actual fact, men need them. End.</t>
-  </si>
-  <si>
-    <t>bachelors. Plesse don't get carried away. You have not said anything bad about your wife. So you have to learn the ropes and date her again, even in marriage. Teach her how to make you need her. Give her your commitment &amp;amp; let her follow your lead. Don't leave her because</t>
-  </si>
-  <si>
-    <t>You all know what is going on in the streets, higher institutions of learning, clubs, hotels etc. Are we saying that all these hook up girls will remain single for life? Are we also saying that they truly cannot make good wives &amp;amp; mothers? If you never met a woman as a Virgin,</t>
+    <t>Please keep all relationship or marriage matters until inec declares the result of the elections. My children deserve a good country to grow in. We need a good country before we can be emotionally balanced to love &amp; be happy in it. End.</t>
+  </si>
+  <si>
+    <t>that we have equal amount of men and women in this community. It clearly says one thing... The pain of heartbreak is more on the one who loves &amp; provides. Women are very unapologetic when they want to move on. And that's how they are created. But you won't listen. End.</t>
+  </si>
+  <si>
+    <t>Married people, What is that thing you and your spouse were always doing together in the early years of your marriage, but now you rarely do it. And your marriage is still as sweet as ever? Me: we couldn't do without eating together, but now, we no send each other 😂😂👇.</t>
+  </si>
+  <si>
+    <t>still alive. Go to him &amp; tell him your concerns. He'll advise you &amp; I'm sure he'll tell you that love is never enough to be with a wife. I also think your wife pampers you so much &amp; you feel it's too good to be true. Wait, until you meet a jezebel, you'll appreciate her. End.</t>
+  </si>
+  <si>
+    <t>Nothing is as disappointing to a lady that's trying to make ends meet, &amp; do so legitimately, seeing another lady that is making ends meet, by just opening her legs. This is why they call such ladies "P. ick Mes" They feel no man wants them. In actual fact, men need them. End.</t>
+  </si>
+  <si>
+    <t>you may just be shooting yourself in the foot. If God thought of them as capable of being on their own, &amp; make decisions that will be of immense help to them, God would not have made men the head of the home &amp; the leader. Today, I talked about triggering the inactive "poison"</t>
+  </si>
+  <si>
+    <t>2. All through his 9 years of marriage, he has been unhappy. He got his wife a job, but she can't bring out N100 to grind beans. She claims she's a feminist, and African women are slaves.</t>
+  </si>
+  <si>
+    <t>commit to it &amp; let her past life be her guide, experience, &amp; motivation not to go back. She'll focus on her marriage &amp; make her own daughters never to be like her. For younger girls, do NOT see this thread as a motivation to continue unabated. You may not be as lucky. End.</t>
+  </si>
+  <si>
+    <t>Things to note on tonight's thread. 1) if you marry her because of the size of her money, you are building on a faulty foundation. 2) if she earns more, remove your eyes from her money. Use yours. 3) if you become jobless &amp; she's stepping in, don't get too comfortable. End.</t>
+  </si>
+  <si>
+    <t>woman must show clear cut difference from a single woman. So for me.. All those men that are married to such women, are either naive, encouraging the wives or the wives are the ones feeding them. I was naive and it took years before I realised my mistake. That's growth. End.</t>
+  </si>
+  <si>
+    <t>After the open discussion tweet for Men last night, do you ladies now see why men don't need your love? It's in heat of an argument, that true feelings are expressed. Men: you don't respect me. Women: you don't love me. Learn to open your minds, when you read from me. End.</t>
+  </si>
+  <si>
+    <t>save you. In one of the DMs in that thread, a man that did not vet or date his wife for long, married into a wealthy family. Under three years of facing financial crisis, his wife left him. In that same DM thread, another man that dated his wife for 7 years, has been jobless</t>
+  </si>
+  <si>
+    <t>bachelors. Plesse don't get carried away. You have not said anything bad about your wife. So you have to learn the ropes and date her again, even in marriage. Teach her how to make you need her. Give her your commitment &amp; let her follow your lead. Don't leave her because</t>
+  </si>
+  <si>
+    <t>I just got one that clearly explains why a man should be "5 steps" ahead of his wife. And why he should not be lazy or relaxed, because his wife is footing the bills. A smart husband who knows that for women, their patience has a shorter lifespan. Interesting DM. End.</t>
+  </si>
+  <si>
+    <t>You all know what is going on in the streets, higher institutions of learning, clubs, hotels etc. Are we saying that all these hook up girls will remain single for life? Are we also saying that they truly cannot make good wives &amp; mothers? If you never met a woman as a Virgin,</t>
   </si>
   <si>
     <t>Let me say this real quick. As a man, you have not found your wife, if you don't consider her "broke". And she will remain your wife, and still be submissive and respectful to you, as long as you still see her as "broke". When a woman feels she's bigger than you?..... End.</t>
@@ -112,37 +169,49 @@
     <t>hate either. You're grooming her into a woman that will serve you and help you fulfil your purpose. No man achieves anything, if he has a bad wife. And sometimes, men enable their wives to be bad. Imagine a woman you married, looking all innocent, loving and caring.</t>
   </si>
   <si>
-    <t>If your girlfriend's female friend is hitting at you, &amp;amp; she knows you're in a relationship with her friend... She knows something about your girlfriend that you don't know. Women will respect the boundaries of their friends, they know respect other women's boundaries. End.</t>
-  </si>
-  <si>
-    <t>Thread on married men that their wives earn more than they do. Are they happy in the marriage? Are their wives still submissive &amp;amp; respectful? 1a. His wife has been showing him pepper since his business crumbled. And he moved into her property.</t>
-  </si>
-  <si>
-    <t>know. And when I make certain decisions, it's not because of selfishness. Or because I don't value &amp;amp; appreciate her. I'm being careful not to turn her into what I'll regret, later. As a man, if you assume that your wife is an adult &amp;amp; can make key decisions on her own,</t>
+    <t>If your girlfriend's female friend is hitting at you, &amp; she knows you're in a relationship with her friend... She knows something about your girlfriend that you don't know. Women will respect the boundaries of their friends, they know respect other women's boundaries. End.</t>
+  </si>
+  <si>
+    <t>Thread on married men that their wives earn more than they do. Are they happy in the marriage? Are their wives still submissive &amp; respectful? 1a. His wife has been showing him pepper since his business crumbled. And he moved into her property.</t>
+  </si>
+  <si>
+    <t>Dear married men, If your wife makes more money than you do, are you happy in your marriage? Does your wife respect &amp; submits to you, like you would expect? If you don't mind, please come to my DM on my back up page to share your experience. Thread from 7pm.</t>
+  </si>
+  <si>
+    <t>know. And when I make certain decisions, it's not because of selfishness. Or because I don't value &amp; appreciate her. I'm being careful not to turn her into what I'll regret, later. As a man, if you assume that your wife is an adult &amp; can make key decisions on her own,</t>
   </si>
   <si>
     <t>Is it not surprising? Ladies who beg men for money few days after meeting them, know that they are hook up girls? So does this truly mean that ladies who say they can't date men who can't take care of them, are really oloshos? What a miracle!. See you tomorrow. End.</t>
   </si>
   <si>
+    <t>losing my mind. Even the men that their wives are currently doing same as my wife, are losing their minds. Despite all the "love", their wives are showing them. They know it's all a matter of time. I don't really like it when myopic minded persons come to argue with me.</t>
+  </si>
+  <si>
+    <t>Open discussion for men. If you're having a quarrel with your gf/wife, and you want to respond to her confrontations. What are you most likely to tell her? 1) don't you have respect? 2) don't you love me anymore? Your comments 👇</t>
+  </si>
+  <si>
     <t>I'm a bit taken aback here. Is the issue being broke or being entitled and hungry? Have you all forgotten that most University girls are broke? Forget the stories about university girls. Are we saying that their fellow students are not dating them? So is it wrong? End.</t>
   </si>
   <si>
+    <t>A man &amp; his wife can have serious misunderstandings, &amp; the next minute, take lovely pictures for SM. Don't pay attention to the pictures. Pay attention to the message. If you're seeing them physically, pay attention to their body language. "i know a very happy couple" End.</t>
+  </si>
+  <si>
     <t>of your wife. I wasn't just playing with words. Your wife will poke her fingers in your eyes, and ask you if it's painful? It doesn't matter for how long you have known her, or for how long you've been married. Always stay 5 steps ahead of her. It's not wickedness. It's not</t>
   </si>
   <si>
-    <t>As a single woman, if you need a child, have one. But don't expect that you'll be immune from the consequences of being a single mother. Except you were a victim of r*pe, you chose to get pregnant &amp;amp; have the baby. You're not the only one having unprotected sex. Grow up! End.</t>
+    <t>As a single woman, if you need a child, have one. But don't expect that you'll be immune from the consequences of being a single mother. Except you were a victim of r*pe, you chose to get pregnant &amp; have the baby. You're not the only one having unprotected sex. Grow up! End.</t>
   </si>
   <si>
     <t>9. He lost his job in 2021. His wife started transferring 250k, out of her 290k salary to him, so he can still be the head. It continued till August 2022, when he got a good job. He promises to give his wife the world.</t>
   </si>
   <si>
-    <t>Then suddenly, she changes into what you can no longer recognize? What happened along the way? Why did she suddenly change? Why is she no longer respectful &amp;amp; submissive like she once was? This is why most men will blame themselves for a failed marriage. Women are quite</t>
+    <t>Then suddenly, she changes into what you can no longer recognize? What happened along the way? Why did she suddenly change? Why is she no longer respectful &amp; submissive like she once was? This is why most men will blame themselves for a failed marriage. Women are quite</t>
   </si>
   <si>
     <t>blame me for it, because they see my wife as a woman who cannot hurt a fly. What they don't understand is that a woman can be perceived as not being able to hurt a fly, because of the man she's under his authority. If you lead your wife the wrong way, you'll be amazed as to</t>
   </si>
   <si>
-    <t>I've been reading comments. All I'll say to men is this. Never wife a KNOWN hoe. If she knows that you know, that she used to be a hoe, &amp;amp; you decide to marry her, it's only a matter of time. When things go south for you, she'll return &amp;amp; still blame you for marrying her.</t>
+    <t>I've been reading comments. All I'll say to men is this. Never wife a KNOWN hoe. If she knows that you know, that she used to be a hoe, &amp; you decide to marry her, it's only a matter of time. When things go south for you, she'll return &amp; still blame you for marrying her.</t>
   </si>
   <si>
     <t>4. He got his wife a job. And ever since she started making money, she has become unruly.</t>
@@ -151,16 +220,31 @@
     <t>A real man goes into a lady's DM, to console her, after Agba has given her wotowoto. With the hope that she'll give him toto. End.</t>
   </si>
   <si>
-    <t>property. She manipulated him &amp;amp; he fell for it. Don't ever think women don't know what they're doing. When you see them come for me, when I make certain tweets, it's all to escape accountability and stop me from exposing their manipulative ways. A woman telling she loves you,</t>
+    <t>And this is what you're experiencing. Now that the love has faded, you want to throw her away? You lie. You did not prepare yourself mentally, for marriage. I also suspect that you are either in your late 20s or early 30s. It also looks like most of your friends are still</t>
+  </si>
+  <si>
+    <t>property. She manipulated him &amp; he fell for it. Don't ever think women don't know what they're doing. When you see them come for me, when I make certain tweets, it's all to escape accountability and stop me from exposing their manipulative ways. A woman telling she loves you,</t>
   </si>
   <si>
     <t>No. You're not going to stay with her, after you get her and knack her. Most men who chase women for that long, are only waiting for their pound of flesh. Especially if the man has been spending on her, while at it.</t>
   </si>
   <si>
-    <t>Open discussion: Can a former prostitute make a good wife &amp;amp; mother? Yes or No and give your reasons 👇.</t>
-  </si>
-  <si>
-    <t>Update on this story. He took my advise and things are looking up for him and his wife. It's the story of the man that slept with their maid. He's also grateful to @talk2veee. Please read 👇</t>
+    <t>the men that shared their stories with me. I don't know them. But all what I've been saying, they've come to validate it. If you discuss theory, no one will validate your teachings. They'll just come to praise you, as your fellow "wokists". And it ends there. You have only</t>
+  </si>
+  <si>
+    <t>Open discussion: Can a former prostitute make a good wife &amp; mother? Yes or No and give your reasons 👇.</t>
+  </si>
+  <si>
+    <t>DM meant for premium Agbafians. But let me just share it here. So all these "my body my choice" woke women will learn. She said she made her husband happy. What does that mean? She gave him snake in the monkey shadow style 😂😂😂😂. Read 👇</t>
+  </si>
+  <si>
+    <t>Update on this story. He took my advise and things are looking up for him and his wife. It's the story of the man that slept with their maid. He's also grateful to . Please read 👇</t>
+  </si>
+  <si>
+    <t>If you're hanging out with random ladies that are dressed skimpy. Just make sure you don't show them my tweets or discuss the tweets. If not, you'll spend plenty money &amp; you will not knack ooo. Don't say it was àgbá that spoilt your show ooo. Act like you don't care. End.</t>
+  </si>
+  <si>
+    <t>You won't wear bra, but when you want to take pics to post on the net, you'll cover the nipple with your fingers. You'll wear skimpy skirts, when you start shaking your bumbum for the net, you'll be using your hands to pull down the skirts so your butts don't show. Idiot. End.</t>
   </si>
   <si>
     <t>10. Ever since he lost his job and business, his wife has made his life a living hell. Read!</t>
@@ -169,21 +253,87 @@
     <t>I've made many mistakes or wrong judgments in my life. But one area I know I did not make the wrong choice, is the choice of my wife. Regardless, I still see my wife as a woman. And if I lose my guard, she will show me that she's a woman. Those who know us, will most likely</t>
   </si>
   <si>
-    <t>very end. Even if she is pretending, let her pretend well. Don't work your butt off, &amp;amp; lose it all just because you want to show love. She'll take advantage of your stupidity. It should always be a carrot &amp;amp; stick approach. I hope we all learn &amp;amp; stop being too weak. End.</t>
-  </si>
-  <si>
-    <t>@ChibuikeIkechu4 As long as the child has a fatherly figure present. But will it be fair to the child to deliberately deny him/her of biological motherly care? No. Even though, I know some people do it.</t>
-  </si>
-  <si>
-    <t>All you feminists &amp;amp; feminised Men that are in this community.. Why are you following me, &amp;amp; why are you afraid to attack me? Are all my almost 170k followers non feminists or feminised men? You know what you're gaining from me. If Dem born your papa well, talk nonsense. End.</t>
-  </si>
-  <si>
-    <t>That DM (to me), appears to be the first DM I'm seeing both men &amp;amp; women coming together as one, to condemn an act. Men are not saying "fear women". And women are not saying "men are scum". Almost everyone has one voice. The thing pain everybody. No pretense. 😂😂😂 End.</t>
+    <t>lady. You negotiate price with her &amp; the next moments, she is with you. Some of them are university girls. They don't need to even go to the streets to display themselves. She comes, you chop &amp; clean mouth. She gets her money &amp; life goes on. Are you saying that another man</t>
+  </si>
+  <si>
+    <t>Then you still don't understand my teachings. Did I say you'll not quarel or fight? That's one of the purpose. Assess yourselves &amp; check where you both have faults. Apologise to each other and continue your relationship if the reason for the quarel is not a red line. End.</t>
+  </si>
+  <si>
+    <t>One hour later... Only 2 screenshots. Even if I ask ladies to post screenshots of men begging them for money, I may not get up 20 screenshots in one hour. That's why I don't spare them when they misbehave. "Agba John Doe is a misogynist" 😂 😂 😂 😂 😂 😂 😂 End.</t>
+  </si>
+  <si>
+    <t>He told a married woman that she's turning him on. I sense he's still a small boy. Remind me to unblock him this weekend.</t>
+  </si>
+  <si>
+    <t>very end. Even if she is pretending, let her pretend well. Don't work your butt off, &amp; lose it all just because you want to show love. She'll take advantage of your stupidity. It should always be a carrot &amp; stick approach. I hope we all learn &amp; stop being too weak. End.</t>
+  </si>
+  <si>
+    <t>You behave like a hoe. You bill him. You tell him that you're bad bitch. You tell him that 5 men have knacked you. Then, he finally gets his chance to knack you. After knacking, you ask him.. "what are we now?" We are pencils in the hands of the creator. End.</t>
+  </si>
+  <si>
+    <t>For those of you that like to ask me about my views on long distance relationship, I wrote this in June last year. Have a read 👇</t>
+  </si>
+  <si>
+    <t>"For just being beautiful, send me your account number". Source: a stupid man. End.</t>
+  </si>
+  <si>
+    <t>Just tell your girlfriend that you prefer her to the lady and that if she leaves, you'll knack the lady and still won't be with her (the one you're flirting with). Your girlfriend is only threatening to leave, because she feels she's not good enough for you. End.</t>
+  </si>
+  <si>
+    <t>They don't think broad. They just wish to use their own "perfect" experience, to argue. They forget that we are talking about humans here. And that as humans, our minds are deep! It's why I will always prove to you all, that my teachings are real. I do not live with any of</t>
+  </si>
+  <si>
+    <t>Hook up girls read that earlier thread and thought Agba has given them a soft landing. 😂😂😂😂😂😂😂😂😂 End.</t>
+  </si>
+  <si>
+    <t>succeeded in making your followers dumber. See me as an imperfect man, blessed by God to do this. I've been consistent in my over 3 years on this platform. Never contradicted myself, for once. If you think I'm here to deceive you, you are just a hater &amp; a myopic being. End.</t>
+  </si>
+  <si>
+    <t>I saw that video. And it was posted by a blog of over 5m followers. Some of these bloggers don't care about the society &amp; are not bothered if they have young impressionable followers. They care about money.</t>
+  </si>
+  <si>
+    <t>Post screenshots of a stupid man that asked for your account number, just because he wants your attention, under this tweet 👇.</t>
+  </si>
+  <si>
+    <t>Women value their nakedness. Any woman that shows it to you privately, can still harm you. Now, imagine the one that doesn't care if the world sees her nakedness? Let me repeat. Once you see any lady that doesn't care if the world sees her sensitive parts, RUN!. End.</t>
+  </si>
+  <si>
+    <t>As long as the child has a fatherly figure present. But will it be fair to the child to deliberately deny him/her of biological motherly care? No. Even though, I know some people do it.</t>
+  </si>
+  <si>
+    <t>always lower your expectations. You will never know the true history of her past life. I know ladies that dated aristos in my university days, that are married. I mean, every weekend was for one aristo or the other. You sit in the comfort of your home, hotel &amp; you chat up a</t>
+  </si>
+  <si>
+    <t>He's 25, and you all know what I mean. Please feel free to advise him.</t>
+  </si>
+  <si>
+    <t>A woman's beauty is in her character or femininity.</t>
+  </si>
+  <si>
+    <t>and she was not happy he did that. Next one he bought, he decided to add her name to it. What happened? They divorced and he lost the property to her. I'm sure she must have told him that she loved him and she felt betrayed by his decision not to jointly add her name to the</t>
+  </si>
+  <si>
+    <t>her, &amp; groomed her well, the longer her patience will last for you. But it will surely have an expiry date. And because she's not asking for a divorce, doesn't mean she's happy playing your roles for you. How much work you have put in, before you married her, is what will</t>
+  </si>
+  <si>
+    <t>All you feminists &amp; feminised Men that are in this community.. Why are you following me, &amp; why are you afraid to attack me? Are all my almost 170k followers non feminists or feminised men? You know what you're gaining from me. If Dem born your papa well, talk nonsense. End.</t>
+  </si>
+  <si>
+    <t>7. He's not married but he's sharing the story of his parents. Read and learn.</t>
+  </si>
+  <si>
+    <t>That DM (to me), appears to be the first DM I'm seeing both men &amp; women coming together as one, to condemn an act. Men are not saying "fear women". And women are not saying "men are scum". Almost everyone has one voice. The thing pain everybody. No pretense. 😂😂😂 End.</t>
+  </si>
+  <si>
+    <t>8. He's not married but he is sharing the story of his parents. Keep reading to learn.</t>
   </si>
   <si>
     <t>She's possibly into hook ups if she: 1) begs for money few days after meeting her 2) turns off data when she's with you 3) lives above her visible means 4) uploads pix from diff hotels 5) posts seductive images online 6) has an "uncle" If this tweet pains you, you're one. End.</t>
   </si>
   <si>
+    <t>until they find themselves in similar situations. They think they're capable of loving men. They are always in their feelings and whatever they feel at the very moment, is what they will believe in. So, many of them reading that thread, will be calling the women in that</t>
+  </si>
+  <si>
     <t>A blog of over 5m followers, thought it "wise" to post video from a lady, advising other ladies to have kids even if they're not married. But thought it wrong to post videos from women, advising other women not to become baby mamas. And you think such blog is helping you? End.</t>
   </si>
   <si>
@@ -196,10 +346,37 @@
     <t>For every wrong move you make on your woman, you'll trigger her inactive "poison". The more you make the wrong move, the closer you're getting to full blown trouble. Always remember... You're living with your best "enemy". End.</t>
   </si>
   <si>
+    <t>I have a question for ladies. How do you feel, when you see your boyfriend using Snapchat filters? Your comments 👇</t>
+  </si>
+  <si>
+    <t>I've written thousands of threads that if people who want to genuinely change the society, share on their large platforms, the society will feel the impact. But hatred &amp; envy won't let them. What they prefer to post is how families will be destroyed &amp; how they make money. End.</t>
+  </si>
+  <si>
+    <t>So you got your gf (that's a student) pregnant twice. The pregnancy disturbed her, &amp; she aborted them. You want to truncate her future, &amp; turn her into a baby mama. Now, you're planning to dump her, because you're not sure she can carry a child? I've no advise for you. End.</t>
+  </si>
+  <si>
+    <t>This one wants to become a baby mama by fire and by force 👇</t>
+  </si>
+  <si>
+    <t>Please watch this video. Do you think it is normal? Yes or No, give your reasons 👇.</t>
+  </si>
+  <si>
     <t>Let me quickly make a correction. A broke girl or lady, is not necessarily someone that is not doing anything. She may be working but may not be making enough, but is content with what she has. And she's not hungry. Space hosts, please take note. Thanks.</t>
   </si>
   <si>
-    <t>I'm beginning to regret why I did not choose to jappa like a lot of my friends and colleagues have done. I've invested so much in this country &amp;amp; the future of my children, but it looks like I'll have to jettison all that, to go start anew in a new country. What a shame. End.</t>
+    <t>I'm beginning to regret why I did not choose to jappa like a lot of my friends and colleagues have done. I've invested so much in this country &amp; the future of my children, but it looks like I'll have to jettison all that, to go start anew in a new country. What a shame. End.</t>
+  </si>
+  <si>
+    <t>Yes, your suspicion is true.</t>
+  </si>
+  <si>
+    <t>Leave story. Post screenshots if you have any. Beggar.</t>
+  </si>
+  <si>
+    <t>Did I ask you? 😒👎</t>
+  </si>
+  <si>
+    <t>At least, they'll not say Agba is biased. In one hour, I can bet I'll not see up to 5 screenshots. I'm still waiting 😂😂😂</t>
   </si>
 </sst>
 </file>
@@ -557,7 +734,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A62"/>
+  <dimension ref="A1:A121"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:1">
@@ -870,6 +1047,301 @@
         <v>61</v>
       </c>
     </row>
+    <row r="63" spans="1:1">
+      <c r="A63" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1">
+      <c r="A64" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1">
+      <c r="A65" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1">
+      <c r="A66" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1">
+      <c r="A67" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1">
+      <c r="A68" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1">
+      <c r="A69" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1">
+      <c r="A70" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1">
+      <c r="A71" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1">
+      <c r="A72" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1">
+      <c r="A73" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1">
+      <c r="A74" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1">
+      <c r="A75" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1">
+      <c r="A76" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1">
+      <c r="A77" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1">
+      <c r="A78" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1">
+      <c r="A79" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1">
+      <c r="A80" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1">
+      <c r="A81" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1">
+      <c r="A82" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1">
+      <c r="A83" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1">
+      <c r="A84" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1">
+      <c r="A85" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1">
+      <c r="A86" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="87" spans="1:1">
+      <c r="A87" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1">
+      <c r="A88" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1">
+      <c r="A89" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1">
+      <c r="A90" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1">
+      <c r="A91" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1">
+      <c r="A92" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="93" spans="1:1">
+      <c r="A93" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1">
+      <c r="A94" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="95" spans="1:1">
+      <c r="A95" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="96" spans="1:1">
+      <c r="A96" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1">
+      <c r="A97" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="98" spans="1:1">
+      <c r="A98" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1">
+      <c r="A99" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="100" spans="1:1">
+      <c r="A100" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="101" spans="1:1">
+      <c r="A101" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="102" spans="1:1">
+      <c r="A102" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="103" spans="1:1">
+      <c r="A103" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="104" spans="1:1">
+      <c r="A104" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="105" spans="1:1">
+      <c r="A105" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="106" spans="1:1">
+      <c r="A106" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="107" spans="1:1">
+      <c r="A107" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="108" spans="1:1">
+      <c r="A108" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="109" spans="1:1">
+      <c r="A109" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="110" spans="1:1">
+      <c r="A110" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="111" spans="1:1">
+      <c r="A111" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="112" spans="1:1">
+      <c r="A112" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="113" spans="1:1">
+      <c r="A113" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="114" spans="1:1">
+      <c r="A114" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="115" spans="1:1">
+      <c r="A115" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="116" spans="1:1">
+      <c r="A116" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="117" spans="1:1">
+      <c r="A117" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="118" spans="1:1">
+      <c r="A118" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="119" spans="1:1">
+      <c r="A119" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="120" spans="1:1">
+      <c r="A120" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="121" spans="1:1">
+      <c r="A121" t="s">
+        <v>120</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>